<commit_message>
Add Lectures 24-27 on floods and droughts; clarify Lecture 21 limiting probability
- L24 Floods I: flood types, ETCCDI indices, annual maxima, return period, risk
- L25 Floods II: Gumbel and log-Pearson III, design floods, climate change, GLOFs
- L26 Droughts I: types of drought, IMD classes, deciles, SPI, SPEI, streamflow index
- L27 Droughts II: theory of runs, drought frequency, warming, management in India
- Worked-example workbooks in data/extremes/
- L21: use P01 = 0.273 throughout and derive the limiting probability step by step
- Update toc, README, CREDITS, intro and Lecture 1 for the new modules
</commit_message>
<xml_diff>
--- a/data/downscaling/lec21/lec21_worked_examples.xlsx
+++ b/data/downscaling/lec21/lec21_worked_examples.xlsx
@@ -20,7 +20,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="0.000"/>
+  </numFmts>
   <fonts count="5">
     <font>
       <name val="Calibri"/>
@@ -68,13 +70,14 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -907,9 +910,7 @@
         </is>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" t="inlineStr"/>
-    </row>
+    <row r="4"/>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
@@ -945,9 +946,7 @@
         </is>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" t="inlineStr"/>
-    </row>
+    <row r="10"/>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
@@ -1686,7 +1685,7 @@
           <t>P11</t>
         </is>
       </c>
-      <c r="J10" s="5">
+      <c r="J10" s="6">
         <f>J4/J8</f>
         <v/>
       </c>
@@ -1729,7 +1728,7 @@
           <t>P10</t>
         </is>
       </c>
-      <c r="J11" s="5">
+      <c r="J11" s="6">
         <f>1-J10</f>
         <v/>
       </c>
@@ -1772,7 +1771,7 @@
           <t>P01</t>
         </is>
       </c>
-      <c r="J12" s="5">
+      <c r="J12" s="6">
         <f>J6/J9</f>
         <v/>
       </c>
@@ -1815,7 +1814,7 @@
           <t>P00</t>
         </is>
       </c>
-      <c r="J13" s="5">
+      <c r="J13" s="6">
         <f>1-J12</f>
         <v/>
       </c>
@@ -1858,7 +1857,7 @@
           <t>P1 (limiting)</t>
         </is>
       </c>
-      <c r="J14" s="5">
+      <c r="J14" s="6">
         <f>J12/(1-J10+J12)</f>
         <v/>
       </c>
@@ -1901,7 +1900,7 @@
           <t>P0</t>
         </is>
       </c>
-      <c r="J15" s="5">
+      <c r="J15" s="6">
         <f>1-J14</f>
         <v/>
       </c>
@@ -1944,7 +1943,7 @@
           <t>check: P11*P1 + P01*P0 - P1</t>
         </is>
       </c>
-      <c r="J16" s="5">
+      <c r="J16" s="6">
         <f>J10*J14+J12*J15-J14</f>
         <v/>
       </c>
@@ -1987,7 +1986,7 @@
           <t>mean wet spell (days)</t>
         </is>
       </c>
-      <c r="J17" s="5">
+      <c r="J17" s="6">
         <f>1/(1-J10)</f>
         <v/>
       </c>
@@ -2030,7 +2029,7 @@
           <t>mean dry spell (days)</t>
         </is>
       </c>
-      <c r="J18" s="5">
+      <c r="J18" s="6">
         <f>1/J12</f>
         <v/>
       </c>
@@ -2073,7 +2072,7 @@
           <t>N1/n (empirical wet fraction)</t>
         </is>
       </c>
-      <c r="J19" s="5">
+      <c r="J19" s="6">
         <f>J2/COUNT(B2:B21)</f>
         <v/>
       </c>
@@ -2116,7 +2115,7 @@
           <t>gamma = P11 - P01</t>
         </is>
       </c>
-      <c r="J20" s="5">
+      <c r="J20" s="6">
         <f>J10-J12</f>
         <v/>
       </c>
@@ -2699,7 +2698,7 @@
           <t>P01</t>
         </is>
       </c>
-      <c r="B2" s="5">
+      <c r="B2" s="6">
         <f>Markov!J12</f>
         <v/>
       </c>
@@ -2715,7 +2714,7 @@
           <t>P11</t>
         </is>
       </c>
-      <c r="B3" s="5">
+      <c r="B3" s="6">
         <f>Markov!J10</f>
         <v/>
       </c>
@@ -2726,7 +2725,7 @@
           <t>P1</t>
         </is>
       </c>
-      <c r="B4" s="5">
+      <c r="B4" s="6">
         <f>Markov!J14</f>
         <v/>
       </c>

</xml_diff>